<commit_message>
Update daily stock screen
</commit_message>
<xml_diff>
--- a/output/daily_screen_20260601.xlsx
+++ b/output/daily_screen_20260601.xlsx
@@ -1306,16 +1306,16 @@
         <v>1</v>
       </c>
       <c r="N7" t="n">
-        <v>37.47320239519422</v>
+        <v>37.47320239521468</v>
       </c>
       <c r="O7" t="n">
-        <v>32.13289453547415</v>
+        <v>32.13289453551437</v>
       </c>
       <c r="P7" t="n">
-        <v>5.34030785972007</v>
+        <v>5.340307859700317</v>
       </c>
       <c r="Q7" t="n">
-        <v>3.239495932092019</v>
+        <v>3.239495932069605</v>
       </c>
       <c r="R7" t="b">
         <v>1</v>
@@ -14123,16 +14123,16 @@
         <v>43.1</v>
       </c>
       <c r="AK7" t="n">
-        <v>37.47320239519422</v>
+        <v>37.47320239521468</v>
       </c>
       <c r="AL7" t="n">
-        <v>32.13289453547415</v>
+        <v>32.13289453551437</v>
       </c>
       <c r="AM7" t="n">
-        <v>5.34030785972007</v>
+        <v>5.340307859700317</v>
       </c>
       <c r="AN7" t="n">
-        <v>3.239495932092019</v>
+        <v>3.239495932069605</v>
       </c>
       <c r="AO7" t="b">
         <v>1</v>

</xml_diff>